<commit_message>
Integrated gradient decent results into Analysis sheet.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/WLMonthlyTemplate.xlsx
+++ b/src/main/resources/static/WLMonthlyTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pf\IntelliJ\ws\aqa\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102E992C-2C7A-4421-9F65-25781F4DA4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F64FBDB1-81BA-4395-88C6-794E8F3F7BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="1095" windowWidth="24645" windowHeight="13185" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4125" yWindow="495" windowWidth="46740" windowHeight="13185" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SNCImport" sheetId="6" r:id="rId1"/>
@@ -980,6 +980,7 @@
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -998,7 +999,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4690,7 +4690,7 @@
         <f t="shared" ref="C21" si="0">10*(C24-C23)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="47" t="s">
+      <c r="G21" s="41" t="s">
         <v>131</v>
       </c>
     </row>
@@ -4887,63 +4887,63 @@
         <v>361</v>
       </c>
       <c r="G3" s="1">
-        <f>ROUND(Data!G3,2)</f>
+        <f>Data!G3</f>
         <v>-1</v>
       </c>
       <c r="H3" s="1">
-        <f>ROUND(Data!H3,2)</f>
+        <f>Data!H3</f>
         <v>-1</v>
       </c>
       <c r="I3" s="1">
-        <f>ROUND(Data!I3,2)</f>
+        <f>Data!I3</f>
         <v>-1</v>
       </c>
       <c r="J3" s="1">
-        <f>ROUND(Data!J3,2)</f>
+        <f>Data!J3</f>
         <v>-1</v>
       </c>
       <c r="K3" s="1">
-        <f>ROUND(Data!K3,2)</f>
+        <f>Data!K3</f>
         <v>-1</v>
       </c>
       <c r="L3" s="1">
-        <f>ROUND(Data!L3,2)</f>
+        <f>Data!L3</f>
         <v>-1</v>
       </c>
       <c r="M3" s="1">
-        <f>ROUND(Data!M3,2)</f>
+        <f>Data!M3</f>
         <v>-1</v>
       </c>
       <c r="N3" s="1">
-        <f>ROUND(Data!N3,2)</f>
+        <f>Data!N3</f>
         <v>-1</v>
       </c>
       <c r="O3" s="1">
-        <f>ROUND(Data!O3,2)</f>
+        <f>Data!O3</f>
         <v>-1</v>
       </c>
       <c r="P3" s="1">
-        <f>ROUND(Data!P3,2)</f>
+        <f>Data!P3</f>
         <v>-1</v>
       </c>
       <c r="Q3" s="1">
-        <f>ROUND(Data!Q3,2)</f>
+        <f>Data!Q3</f>
         <v>-1</v>
       </c>
       <c r="R3" s="1">
-        <f>ROUND(Data!R3,2)</f>
+        <f>Data!R3</f>
         <v>-1</v>
       </c>
       <c r="S3" s="1">
-        <f>ROUND(Data!S3,2)</f>
+        <f>Data!S3</f>
         <v>-1</v>
       </c>
       <c r="T3" s="1">
-        <f>ROUND(Data!T3,2)</f>
+        <f>Data!T3</f>
         <v>-1</v>
       </c>
       <c r="U3" s="1">
-        <f>ROUND(Data!U3,2)</f>
+        <f>Data!U3</f>
         <v>-1</v>
       </c>
       <c r="V3" t="str">
@@ -4977,63 +4977,63 @@
         <v>361</v>
       </c>
       <c r="G4" s="1">
-        <f>ROUND(Data!G4,2)</f>
+        <f>Data!G4</f>
         <v>-1</v>
       </c>
       <c r="H4" s="1">
-        <f>ROUND(Data!H4,2)</f>
+        <f>Data!H4</f>
         <v>-1</v>
       </c>
       <c r="I4" s="1">
-        <f>ROUND(Data!I4,2)</f>
+        <f>Data!I4</f>
         <v>-1</v>
       </c>
       <c r="J4" s="1">
-        <f>ROUND(Data!J4,2)</f>
+        <f>Data!J4</f>
         <v>-1</v>
       </c>
       <c r="K4" s="1">
-        <f>ROUND(Data!K4,2)</f>
+        <f>Data!K4</f>
         <v>-1</v>
       </c>
       <c r="L4" s="1">
-        <f>ROUND(Data!L4,2)</f>
+        <f>Data!L4</f>
         <v>-1</v>
       </c>
       <c r="M4" s="1">
-        <f>ROUND(Data!M4,2)</f>
+        <f>Data!M4</f>
         <v>-1</v>
       </c>
       <c r="N4" s="1">
-        <f>ROUND(Data!N4,2)</f>
+        <f>Data!N4</f>
         <v>-1</v>
       </c>
       <c r="O4" s="1">
-        <f>ROUND(Data!O4,2)</f>
+        <f>Data!O4</f>
         <v>-1</v>
       </c>
       <c r="P4" s="1">
-        <f>ROUND(Data!P4,2)</f>
+        <f>Data!P4</f>
         <v>-1</v>
       </c>
       <c r="Q4" s="1">
-        <f>ROUND(Data!Q4,2)</f>
+        <f>Data!Q4</f>
         <v>-1</v>
       </c>
       <c r="R4" s="1">
-        <f>ROUND(Data!R4,2)</f>
+        <f>Data!R4</f>
         <v>-1</v>
       </c>
       <c r="S4" s="1">
-        <f>ROUND(Data!S4,2)</f>
+        <f>Data!S4</f>
         <v>-1</v>
       </c>
       <c r="T4" s="1">
-        <f>ROUND(Data!T4,2)</f>
+        <f>Data!T4</f>
         <v>-1</v>
       </c>
       <c r="U4" s="1">
-        <f>ROUND(Data!U4,2)</f>
+        <f>Data!U4</f>
         <v>-1</v>
       </c>
       <c r="V4" t="str">
@@ -5067,63 +5067,63 @@
         <v>361</v>
       </c>
       <c r="G5" s="1">
-        <f>ROUND(Data!G5,2)</f>
+        <f>Data!G5</f>
         <v>-1</v>
       </c>
       <c r="H5" s="1">
-        <f>ROUND(Data!H5,2)</f>
+        <f>Data!H5</f>
         <v>-1</v>
       </c>
       <c r="I5" s="1">
-        <f>ROUND(Data!I5,2)</f>
+        <f>Data!I5</f>
         <v>-1</v>
       </c>
       <c r="J5" s="1">
-        <f>ROUND(Data!J5,2)</f>
+        <f>Data!J5</f>
         <v>-1</v>
       </c>
       <c r="K5" s="1">
-        <f>ROUND(Data!K5,2)</f>
+        <f>Data!K5</f>
         <v>-1</v>
       </c>
       <c r="L5" s="1">
-        <f>ROUND(Data!L5,2)</f>
+        <f>Data!L5</f>
         <v>-1</v>
       </c>
       <c r="M5" s="1">
-        <f>ROUND(Data!M5,2)</f>
+        <f>Data!M5</f>
         <v>-1</v>
       </c>
       <c r="N5" s="1">
-        <f>ROUND(Data!N5,2)</f>
+        <f>Data!N5</f>
         <v>-1</v>
       </c>
       <c r="O5" s="1">
-        <f>ROUND(Data!O5,2)</f>
+        <f>Data!O5</f>
         <v>-1</v>
       </c>
       <c r="P5" s="1">
-        <f>ROUND(Data!P5,2)</f>
+        <f>Data!P5</f>
         <v>-1</v>
       </c>
       <c r="Q5" s="1">
-        <f>ROUND(Data!Q5,2)</f>
+        <f>Data!Q5</f>
         <v>-1</v>
       </c>
       <c r="R5" s="1">
-        <f>ROUND(Data!R5,2)</f>
+        <f>Data!R5</f>
         <v>-1</v>
       </c>
       <c r="S5" s="1">
-        <f>ROUND(Data!S5,2)</f>
+        <f>Data!S5</f>
         <v>-1</v>
       </c>
       <c r="T5" s="1">
-        <f>ROUND(Data!T5,2)</f>
+        <f>Data!T5</f>
         <v>-1</v>
       </c>
       <c r="U5" s="1">
-        <f>ROUND(Data!U5,2)</f>
+        <f>Data!U5</f>
         <v>-1</v>
       </c>
       <c r="V5" t="str">
@@ -5157,63 +5157,63 @@
         <v>361</v>
       </c>
       <c r="G6" s="1">
-        <f>ROUND(Data!G6,2)</f>
+        <f>Data!G6</f>
         <v>-1</v>
       </c>
       <c r="H6" s="1">
-        <f>ROUND(Data!H6,2)</f>
+        <f>Data!H6</f>
         <v>-1</v>
       </c>
       <c r="I6" s="1">
-        <f>ROUND(Data!I6,2)</f>
+        <f>Data!I6</f>
         <v>-1</v>
       </c>
       <c r="J6" s="1">
-        <f>ROUND(Data!J6,2)</f>
+        <f>Data!J6</f>
         <v>-1</v>
       </c>
       <c r="K6" s="1">
-        <f>ROUND(Data!K6,2)</f>
+        <f>Data!K6</f>
         <v>-1</v>
       </c>
       <c r="L6" s="1">
-        <f>ROUND(Data!L6,2)</f>
+        <f>Data!L6</f>
         <v>-1</v>
       </c>
       <c r="M6" s="1">
-        <f>ROUND(Data!M6,2)</f>
+        <f>Data!M6</f>
         <v>-1</v>
       </c>
       <c r="N6" s="1">
-        <f>ROUND(Data!N6,2)</f>
+        <f>Data!N6</f>
         <v>-1</v>
       </c>
       <c r="O6" s="1">
-        <f>ROUND(Data!O6,2)</f>
+        <f>Data!O6</f>
         <v>-1</v>
       </c>
       <c r="P6" s="1">
-        <f>ROUND(Data!P6,2)</f>
+        <f>Data!P6</f>
         <v>-1</v>
       </c>
       <c r="Q6" s="1">
-        <f>ROUND(Data!Q6,2)</f>
+        <f>Data!Q6</f>
         <v>-1</v>
       </c>
       <c r="R6" s="1">
-        <f>ROUND(Data!R6,2)</f>
+        <f>Data!R6</f>
         <v>-1</v>
       </c>
       <c r="S6" s="1">
-        <f>ROUND(Data!S6,2)</f>
+        <f>Data!S6</f>
         <v>-1</v>
       </c>
       <c r="T6" s="1">
-        <f>ROUND(Data!T6,2)</f>
+        <f>Data!T6</f>
         <v>-1</v>
       </c>
       <c r="U6" s="1">
-        <f>ROUND(Data!U6,2)</f>
+        <f>Data!U6</f>
         <v>-1</v>
       </c>
       <c r="V6" t="str">
@@ -5247,63 +5247,63 @@
         <v>361</v>
       </c>
       <c r="G7" s="1">
-        <f>ROUND(Data!G7,2)</f>
+        <f>Data!G7</f>
         <v>-1</v>
       </c>
       <c r="H7" s="1">
-        <f>ROUND(Data!H7,2)</f>
+        <f>Data!H7</f>
         <v>-1</v>
       </c>
       <c r="I7" s="1">
-        <f>ROUND(Data!I7,2)</f>
+        <f>Data!I7</f>
         <v>-1</v>
       </c>
       <c r="J7" s="1">
-        <f>ROUND(Data!J7,2)</f>
+        <f>Data!J7</f>
         <v>-1</v>
       </c>
       <c r="K7" s="1">
-        <f>ROUND(Data!K7,2)</f>
+        <f>Data!K7</f>
         <v>-1</v>
       </c>
       <c r="L7" s="1">
-        <f>ROUND(Data!L7,2)</f>
+        <f>Data!L7</f>
         <v>-1</v>
       </c>
       <c r="M7" s="1">
-        <f>ROUND(Data!M7,2)</f>
+        <f>Data!M7</f>
         <v>-1</v>
       </c>
       <c r="N7" s="1">
-        <f>ROUND(Data!N7,2)</f>
+        <f>Data!N7</f>
         <v>-1</v>
       </c>
       <c r="O7" s="1">
-        <f>ROUND(Data!O7,2)</f>
+        <f>Data!O7</f>
         <v>-1</v>
       </c>
       <c r="P7" s="1">
-        <f>ROUND(Data!P7,2)</f>
+        <f>Data!P7</f>
         <v>-1</v>
       </c>
       <c r="Q7" s="1">
-        <f>ROUND(Data!Q7,2)</f>
+        <f>Data!Q7</f>
         <v>-1</v>
       </c>
       <c r="R7" s="1">
-        <f>ROUND(Data!R7,2)</f>
+        <f>Data!R7</f>
         <v>-1</v>
       </c>
       <c r="S7" s="1">
-        <f>ROUND(Data!S7,2)</f>
+        <f>Data!S7</f>
         <v>-1</v>
       </c>
       <c r="T7" s="1">
-        <f>ROUND(Data!T7,2)</f>
+        <f>Data!T7</f>
         <v>-1</v>
       </c>
       <c r="U7" s="1">
-        <f>ROUND(Data!U7,2)</f>
+        <f>Data!U7</f>
         <v>-1</v>
       </c>
       <c r="V7" t="str">
@@ -5337,63 +5337,63 @@
         <v>361</v>
       </c>
       <c r="G8" s="1">
-        <f>ROUND(Data!G8,2)</f>
+        <f>Data!G8</f>
         <v>-1</v>
       </c>
       <c r="H8" s="1">
-        <f>ROUND(Data!H8,2)</f>
+        <f>Data!H8</f>
         <v>-1</v>
       </c>
       <c r="I8" s="1">
-        <f>ROUND(Data!I8,2)</f>
+        <f>Data!I8</f>
         <v>-1</v>
       </c>
       <c r="J8" s="1">
-        <f>ROUND(Data!J8,2)</f>
+        <f>Data!J8</f>
         <v>-1</v>
       </c>
       <c r="K8" s="1">
-        <f>ROUND(Data!K8,2)</f>
+        <f>Data!K8</f>
         <v>-1</v>
       </c>
       <c r="L8" s="1">
-        <f>ROUND(Data!L8,2)</f>
+        <f>Data!L8</f>
         <v>-1</v>
       </c>
       <c r="M8" s="1">
-        <f>ROUND(Data!M8,2)</f>
+        <f>Data!M8</f>
         <v>-1</v>
       </c>
       <c r="N8" s="1">
-        <f>ROUND(Data!N8,2)</f>
+        <f>Data!N8</f>
         <v>-1</v>
       </c>
       <c r="O8" s="1">
-        <f>ROUND(Data!O8,2)</f>
+        <f>Data!O8</f>
         <v>-1</v>
       </c>
       <c r="P8" s="1">
-        <f>ROUND(Data!P8,2)</f>
+        <f>Data!P8</f>
         <v>-1</v>
       </c>
       <c r="Q8" s="1">
-        <f>ROUND(Data!Q8,2)</f>
+        <f>Data!Q8</f>
         <v>-1</v>
       </c>
       <c r="R8" s="1">
-        <f>ROUND(Data!R8,2)</f>
+        <f>Data!R8</f>
         <v>-1</v>
       </c>
       <c r="S8" s="1">
-        <f>ROUND(Data!S8,2)</f>
+        <f>Data!S8</f>
         <v>-1</v>
       </c>
       <c r="T8" s="1">
-        <f>ROUND(Data!T8,2)</f>
+        <f>Data!T8</f>
         <v>-1</v>
       </c>
       <c r="U8" s="1">
-        <f>ROUND(Data!U8,2)</f>
+        <f>Data!U8</f>
         <v>-1</v>
       </c>
       <c r="V8" t="str">
@@ -5427,63 +5427,63 @@
         <v>361</v>
       </c>
       <c r="G9" s="1">
-        <f>ROUND(Data!G9,2)</f>
+        <f>Data!G9</f>
         <v>-1</v>
       </c>
       <c r="H9" s="1">
-        <f>ROUND(Data!H9,2)</f>
+        <f>Data!H9</f>
         <v>-1</v>
       </c>
       <c r="I9" s="1">
-        <f>ROUND(Data!I9,2)</f>
+        <f>Data!I9</f>
         <v>-1</v>
       </c>
       <c r="J9" s="1">
-        <f>ROUND(Data!J9,2)</f>
+        <f>Data!J9</f>
         <v>-1</v>
       </c>
       <c r="K9" s="1">
-        <f>ROUND(Data!K9,2)</f>
+        <f>Data!K9</f>
         <v>-1</v>
       </c>
       <c r="L9" s="1">
-        <f>ROUND(Data!L9,2)</f>
+        <f>Data!L9</f>
         <v>-1</v>
       </c>
       <c r="M9" s="1">
-        <f>ROUND(Data!M9,2)</f>
+        <f>Data!M9</f>
         <v>-1</v>
       </c>
       <c r="N9" s="1">
-        <f>ROUND(Data!N9,2)</f>
+        <f>Data!N9</f>
         <v>-1</v>
       </c>
       <c r="O9" s="1">
-        <f>ROUND(Data!O9,2)</f>
+        <f>Data!O9</f>
         <v>-1</v>
       </c>
       <c r="P9" s="1">
-        <f>ROUND(Data!P9,2)</f>
+        <f>Data!P9</f>
         <v>-1</v>
       </c>
       <c r="Q9" s="1">
-        <f>ROUND(Data!Q9,2)</f>
+        <f>Data!Q9</f>
         <v>-1</v>
       </c>
       <c r="R9" s="1">
-        <f>ROUND(Data!R9,2)</f>
+        <f>Data!R9</f>
         <v>-1</v>
       </c>
       <c r="S9" s="1">
-        <f>ROUND(Data!S9,2)</f>
+        <f>Data!S9</f>
         <v>-1</v>
       </c>
       <c r="T9" s="1">
-        <f>ROUND(Data!T9,2)</f>
+        <f>Data!T9</f>
         <v>-1</v>
       </c>
       <c r="U9" s="1">
-        <f>ROUND(Data!U9,2)</f>
+        <f>Data!U9</f>
         <v>-1</v>
       </c>
       <c r="V9" t="str">
@@ -5517,63 +5517,63 @@
         <v>361</v>
       </c>
       <c r="G10" s="1">
-        <f>ROUND(Data!G10,2)</f>
+        <f>Data!G10</f>
         <v>-1</v>
       </c>
       <c r="H10" s="1">
-        <f>ROUND(Data!H10,2)</f>
+        <f>Data!H10</f>
         <v>-1</v>
       </c>
       <c r="I10" s="1">
-        <f>ROUND(Data!I10,2)</f>
+        <f>Data!I10</f>
         <v>-1</v>
       </c>
       <c r="J10" s="1">
-        <f>ROUND(Data!J10,2)</f>
+        <f>Data!J10</f>
         <v>-1</v>
       </c>
       <c r="K10" s="1">
-        <f>ROUND(Data!K10,2)</f>
+        <f>Data!K10</f>
         <v>-1</v>
       </c>
       <c r="L10" s="1">
-        <f>ROUND(Data!L10,2)</f>
+        <f>Data!L10</f>
         <v>-1</v>
       </c>
       <c r="M10" s="1">
-        <f>ROUND(Data!M10,2)</f>
+        <f>Data!M10</f>
         <v>-1</v>
       </c>
       <c r="N10" s="1">
-        <f>ROUND(Data!N10,2)</f>
+        <f>Data!N10</f>
         <v>-1</v>
       </c>
       <c r="O10" s="1">
-        <f>ROUND(Data!O10,2)</f>
+        <f>Data!O10</f>
         <v>-1</v>
       </c>
       <c r="P10" s="1">
-        <f>ROUND(Data!P10,2)</f>
+        <f>Data!P10</f>
         <v>-1</v>
       </c>
       <c r="Q10" s="1">
-        <f>ROUND(Data!Q10,2)</f>
+        <f>Data!Q10</f>
         <v>-1</v>
       </c>
       <c r="R10" s="1">
-        <f>ROUND(Data!R10,2)</f>
+        <f>Data!R10</f>
         <v>-1</v>
       </c>
       <c r="S10" s="1">
-        <f>ROUND(Data!S10,2)</f>
+        <f>Data!S10</f>
         <v>-1</v>
       </c>
       <c r="T10" s="1">
-        <f>ROUND(Data!T10,2)</f>
+        <f>Data!T10</f>
         <v>-1</v>
       </c>
       <c r="U10" s="1">
-        <f>ROUND(Data!U10,2)</f>
+        <f>Data!U10</f>
         <v>-1</v>
       </c>
       <c r="V10" t="str">
@@ -5607,63 +5607,63 @@
         <v>361</v>
       </c>
       <c r="G11" s="1">
-        <f>ROUND(Data!G11,2)</f>
+        <f>Data!G11</f>
         <v>-1</v>
       </c>
       <c r="H11" s="1">
-        <f>ROUND(Data!H11,2)</f>
+        <f>Data!H11</f>
         <v>-1</v>
       </c>
       <c r="I11" s="1">
-        <f>ROUND(Data!I11,2)</f>
+        <f>Data!I11</f>
         <v>-1</v>
       </c>
       <c r="J11" s="1">
-        <f>ROUND(Data!J11,2)</f>
+        <f>Data!J11</f>
         <v>-1</v>
       </c>
       <c r="K11" s="1">
-        <f>ROUND(Data!K11,2)</f>
+        <f>Data!K11</f>
         <v>-1</v>
       </c>
       <c r="L11" s="1">
-        <f>ROUND(Data!L11,2)</f>
+        <f>Data!L11</f>
         <v>-1</v>
       </c>
       <c r="M11" s="1">
-        <f>ROUND(Data!M11,2)</f>
+        <f>Data!M11</f>
         <v>-1</v>
       </c>
       <c r="N11" s="1">
-        <f>ROUND(Data!N11,2)</f>
+        <f>Data!N11</f>
         <v>-1</v>
       </c>
       <c r="O11" s="1">
-        <f>ROUND(Data!O11,2)</f>
+        <f>Data!O11</f>
         <v>-1</v>
       </c>
       <c r="P11" s="1">
-        <f>ROUND(Data!P11,2)</f>
+        <f>Data!P11</f>
         <v>-1</v>
       </c>
       <c r="Q11" s="1">
-        <f>ROUND(Data!Q11,2)</f>
+        <f>Data!Q11</f>
         <v>-1</v>
       </c>
       <c r="R11" s="1">
-        <f>ROUND(Data!R11,2)</f>
+        <f>Data!R11</f>
         <v>-1</v>
       </c>
       <c r="S11" s="1">
-        <f>ROUND(Data!S11,2)</f>
+        <f>Data!S11</f>
         <v>-1</v>
       </c>
       <c r="T11" s="1">
-        <f>ROUND(Data!T11,2)</f>
+        <f>Data!T11</f>
         <v>-1</v>
       </c>
       <c r="U11" s="1">
-        <f>ROUND(Data!U11,2)</f>
+        <f>Data!U11</f>
         <v>-1</v>
       </c>
       <c r="V11" t="str">
@@ -5697,63 +5697,63 @@
         <v>361</v>
       </c>
       <c r="G12" s="1">
-        <f>ROUND(Data!G12,2)</f>
+        <f>Data!G12</f>
         <v>-1</v>
       </c>
       <c r="H12" s="1">
-        <f>ROUND(Data!H12,2)</f>
+        <f>Data!H12</f>
         <v>-1</v>
       </c>
       <c r="I12" s="1">
-        <f>ROUND(Data!I12,2)</f>
+        <f>Data!I12</f>
         <v>-1</v>
       </c>
       <c r="J12" s="1">
-        <f>ROUND(Data!J12,2)</f>
+        <f>Data!J12</f>
         <v>-1</v>
       </c>
       <c r="K12" s="1">
-        <f>ROUND(Data!K12,2)</f>
+        <f>Data!K12</f>
         <v>-1</v>
       </c>
       <c r="L12" s="1">
-        <f>ROUND(Data!L12,2)</f>
+        <f>Data!L12</f>
         <v>-1</v>
       </c>
       <c r="M12" s="1">
-        <f>ROUND(Data!M12,2)</f>
+        <f>Data!M12</f>
         <v>-1</v>
       </c>
       <c r="N12" s="1">
-        <f>ROUND(Data!N12,2)</f>
+        <f>Data!N12</f>
         <v>-1</v>
       </c>
       <c r="O12" s="1">
-        <f>ROUND(Data!O12,2)</f>
+        <f>Data!O12</f>
         <v>-1</v>
       </c>
       <c r="P12" s="1">
-        <f>ROUND(Data!P12,2)</f>
+        <f>Data!P12</f>
         <v>-1</v>
       </c>
       <c r="Q12" s="1">
-        <f>ROUND(Data!Q12,2)</f>
+        <f>Data!Q12</f>
         <v>-1</v>
       </c>
       <c r="R12" s="1">
-        <f>ROUND(Data!R12,2)</f>
+        <f>Data!R12</f>
         <v>-1</v>
       </c>
       <c r="S12" s="1">
-        <f>ROUND(Data!S12,2)</f>
+        <f>Data!S12</f>
         <v>-1</v>
       </c>
       <c r="T12" s="1">
-        <f>ROUND(Data!T12,2)</f>
+        <f>Data!T12</f>
         <v>-1</v>
       </c>
       <c r="U12" s="1">
-        <f>ROUND(Data!U12,2)</f>
+        <f>Data!U12</f>
         <v>-1</v>
       </c>
       <c r="V12" t="str">
@@ -5787,63 +5787,63 @@
         <v>361</v>
       </c>
       <c r="G13" s="1">
-        <f>ROUND(Data!G13,2)</f>
+        <f>Data!G13</f>
         <v>-1</v>
       </c>
       <c r="H13" s="1">
-        <f>ROUND(Data!H13,2)</f>
+        <f>Data!H13</f>
         <v>-1</v>
       </c>
       <c r="I13" s="1">
-        <f>ROUND(Data!I13,2)</f>
+        <f>Data!I13</f>
         <v>-1</v>
       </c>
       <c r="J13" s="1">
-        <f>ROUND(Data!J13,2)</f>
+        <f>Data!J13</f>
         <v>-1</v>
       </c>
       <c r="K13" s="1">
-        <f>ROUND(Data!K13,2)</f>
+        <f>Data!K13</f>
         <v>-1</v>
       </c>
       <c r="L13" s="1">
-        <f>ROUND(Data!L13,2)</f>
+        <f>Data!L13</f>
         <v>-1</v>
       </c>
       <c r="M13" s="1">
-        <f>ROUND(Data!M13,2)</f>
+        <f>Data!M13</f>
         <v>-1</v>
       </c>
       <c r="N13" s="1">
-        <f>ROUND(Data!N13,2)</f>
+        <f>Data!N13</f>
         <v>-1</v>
       </c>
       <c r="O13" s="1">
-        <f>ROUND(Data!O13,2)</f>
+        <f>Data!O13</f>
         <v>-1</v>
       </c>
       <c r="P13" s="1">
-        <f>ROUND(Data!P13,2)</f>
+        <f>Data!P13</f>
         <v>-1</v>
       </c>
       <c r="Q13" s="1">
-        <f>ROUND(Data!Q13,2)</f>
+        <f>Data!Q13</f>
         <v>-1</v>
       </c>
       <c r="R13" s="1">
-        <f>ROUND(Data!R13,2)</f>
+        <f>Data!R13</f>
         <v>-1</v>
       </c>
       <c r="S13" s="1">
-        <f>ROUND(Data!S13,2)</f>
+        <f>Data!S13</f>
         <v>-1</v>
       </c>
       <c r="T13" s="1">
-        <f>ROUND(Data!T13,2)</f>
+        <f>Data!T13</f>
         <v>-1</v>
       </c>
       <c r="U13" s="1">
-        <f>ROUND(Data!U13,2)</f>
+        <f>Data!U13</f>
         <v>-1</v>
       </c>
       <c r="V13" t="str">
@@ -5877,63 +5877,63 @@
         <v>361</v>
       </c>
       <c r="G14" s="1">
-        <f>ROUND(Data!G14,2)</f>
+        <f>Data!G14</f>
         <v>-1</v>
       </c>
       <c r="H14" s="1">
-        <f>ROUND(Data!H14,2)</f>
+        <f>Data!H14</f>
         <v>-1</v>
       </c>
       <c r="I14" s="1">
-        <f>ROUND(Data!I14,2)</f>
+        <f>Data!I14</f>
         <v>-1</v>
       </c>
       <c r="J14" s="1">
-        <f>ROUND(Data!J14,2)</f>
+        <f>Data!J14</f>
         <v>-1</v>
       </c>
       <c r="K14" s="1">
-        <f>ROUND(Data!K14,2)</f>
+        <f>Data!K14</f>
         <v>-1</v>
       </c>
       <c r="L14" s="1">
-        <f>ROUND(Data!L14,2)</f>
+        <f>Data!L14</f>
         <v>-1</v>
       </c>
       <c r="M14" s="1">
-        <f>ROUND(Data!M14,2)</f>
+        <f>Data!M14</f>
         <v>-1</v>
       </c>
       <c r="N14" s="1">
-        <f>ROUND(Data!N14,2)</f>
+        <f>Data!N14</f>
         <v>-1</v>
       </c>
       <c r="O14" s="1">
-        <f>ROUND(Data!O14,2)</f>
+        <f>Data!O14</f>
         <v>-1</v>
       </c>
       <c r="P14" s="1">
-        <f>ROUND(Data!P14,2)</f>
+        <f>Data!P14</f>
         <v>-1</v>
       </c>
       <c r="Q14" s="1">
-        <f>ROUND(Data!Q14,2)</f>
+        <f>Data!Q14</f>
         <v>-1</v>
       </c>
       <c r="R14" s="1">
-        <f>ROUND(Data!R14,2)</f>
+        <f>Data!R14</f>
         <v>-1</v>
       </c>
       <c r="S14" s="1">
-        <f>ROUND(Data!S14,2)</f>
+        <f>Data!S14</f>
         <v>-1</v>
       </c>
       <c r="T14" s="1">
-        <f>ROUND(Data!T14,2)</f>
+        <f>Data!T14</f>
         <v>-1</v>
       </c>
       <c r="U14" s="1">
-        <f>ROUND(Data!U14,2)</f>
+        <f>Data!U14</f>
         <v>-1</v>
       </c>
       <c r="V14" t="str">
@@ -5967,63 +5967,63 @@
         <v>361</v>
       </c>
       <c r="G15" s="1">
-        <f>ROUND(Data!G15,2)</f>
+        <f>Data!G15</f>
         <v>-1</v>
       </c>
       <c r="H15" s="1">
-        <f>ROUND(Data!H15,2)</f>
+        <f>Data!H15</f>
         <v>-1</v>
       </c>
       <c r="I15" s="1">
-        <f>ROUND(Data!I15,2)</f>
+        <f>Data!I15</f>
         <v>-1</v>
       </c>
       <c r="J15" s="1">
-        <f>ROUND(Data!J15,2)</f>
+        <f>Data!J15</f>
         <v>-1</v>
       </c>
       <c r="K15" s="1">
-        <f>ROUND(Data!K15,2)</f>
+        <f>Data!K15</f>
         <v>-1</v>
       </c>
       <c r="L15" s="1">
-        <f>ROUND(Data!L15,2)</f>
+        <f>Data!L15</f>
         <v>-1</v>
       </c>
       <c r="M15" s="1">
-        <f>ROUND(Data!M15,2)</f>
+        <f>Data!M15</f>
         <v>-1</v>
       </c>
       <c r="N15" s="1">
-        <f>ROUND(Data!N15,2)</f>
+        <f>Data!N15</f>
         <v>-1</v>
       </c>
       <c r="O15" s="1">
-        <f>ROUND(Data!O15,2)</f>
+        <f>Data!O15</f>
         <v>-1</v>
       </c>
       <c r="P15" s="1">
-        <f>ROUND(Data!P15,2)</f>
+        <f>Data!P15</f>
         <v>-1</v>
       </c>
       <c r="Q15" s="1">
-        <f>ROUND(Data!Q15,2)</f>
+        <f>Data!Q15</f>
         <v>-1</v>
       </c>
       <c r="R15" s="1">
-        <f>ROUND(Data!R15,2)</f>
+        <f>Data!R15</f>
         <v>-1</v>
       </c>
       <c r="S15" s="1">
-        <f>ROUND(Data!S15,2)</f>
+        <f>Data!S15</f>
         <v>-1</v>
       </c>
       <c r="T15" s="1">
-        <f>ROUND(Data!T15,2)</f>
+        <f>Data!T15</f>
         <v>-1</v>
       </c>
       <c r="U15" s="1">
-        <f>ROUND(Data!U15,2)</f>
+        <f>Data!U15</f>
         <v>-1</v>
       </c>
       <c r="V15" t="str">
@@ -6057,63 +6057,63 @@
         <v>361</v>
       </c>
       <c r="G16" s="1">
-        <f>ROUND(Data!G16,2)</f>
+        <f>Data!G16</f>
         <v>-1</v>
       </c>
       <c r="H16" s="1">
-        <f>ROUND(Data!H16,2)</f>
+        <f>Data!H16</f>
         <v>-1</v>
       </c>
       <c r="I16" s="1">
-        <f>ROUND(Data!I16,2)</f>
+        <f>Data!I16</f>
         <v>-1</v>
       </c>
       <c r="J16" s="1">
-        <f>ROUND(Data!J16,2)</f>
+        <f>Data!J16</f>
         <v>-1</v>
       </c>
       <c r="K16" s="1">
-        <f>ROUND(Data!K16,2)</f>
+        <f>Data!K16</f>
         <v>-1</v>
       </c>
       <c r="L16" s="1">
-        <f>ROUND(Data!L16,2)</f>
+        <f>Data!L16</f>
         <v>-1</v>
       </c>
       <c r="M16" s="1">
-        <f>ROUND(Data!M16,2)</f>
+        <f>Data!M16</f>
         <v>-1</v>
       </c>
       <c r="N16" s="1">
-        <f>ROUND(Data!N16,2)</f>
+        <f>Data!N16</f>
         <v>-1</v>
       </c>
       <c r="O16" s="1">
-        <f>ROUND(Data!O16,2)</f>
+        <f>Data!O16</f>
         <v>-1</v>
       </c>
       <c r="P16" s="1">
-        <f>ROUND(Data!P16,2)</f>
+        <f>Data!P16</f>
         <v>-1</v>
       </c>
       <c r="Q16" s="1">
-        <f>ROUND(Data!Q16,2)</f>
+        <f>Data!Q16</f>
         <v>-1</v>
       </c>
       <c r="R16" s="1">
-        <f>ROUND(Data!R16,2)</f>
+        <f>Data!R16</f>
         <v>-1</v>
       </c>
       <c r="S16" s="1">
-        <f>ROUND(Data!S16,2)</f>
+        <f>Data!S16</f>
         <v>-1</v>
       </c>
       <c r="T16" s="1">
-        <f>ROUND(Data!T16,2)</f>
+        <f>Data!T16</f>
         <v>-1</v>
       </c>
       <c r="U16" s="1">
-        <f>ROUND(Data!U16,2)</f>
+        <f>Data!U16</f>
         <v>-1</v>
       </c>
       <c r="V16" t="str">
@@ -6147,63 +6147,63 @@
         <v>361</v>
       </c>
       <c r="G17" s="1">
-        <f>ROUND(Data!G17,2)</f>
+        <f>Data!G17</f>
         <v>-1</v>
       </c>
       <c r="H17" s="1">
-        <f>ROUND(Data!H17,2)</f>
+        <f>Data!H17</f>
         <v>-1</v>
       </c>
       <c r="I17" s="1">
-        <f>ROUND(Data!I17,2)</f>
+        <f>Data!I17</f>
         <v>-1</v>
       </c>
       <c r="J17" s="1">
-        <f>ROUND(Data!J17,2)</f>
+        <f>Data!J17</f>
         <v>-1</v>
       </c>
       <c r="K17" s="1">
-        <f>ROUND(Data!K17,2)</f>
+        <f>Data!K17</f>
         <v>-1</v>
       </c>
       <c r="L17" s="1">
-        <f>ROUND(Data!L17,2)</f>
+        <f>Data!L17</f>
         <v>-1</v>
       </c>
       <c r="M17" s="1">
-        <f>ROUND(Data!M17,2)</f>
+        <f>Data!M17</f>
         <v>-1</v>
       </c>
       <c r="N17" s="1">
-        <f>ROUND(Data!N17,2)</f>
+        <f>Data!N17</f>
         <v>-1</v>
       </c>
       <c r="O17" s="1">
-        <f>ROUND(Data!O17,2)</f>
+        <f>Data!O17</f>
         <v>-1</v>
       </c>
       <c r="P17" s="1">
-        <f>ROUND(Data!P17,2)</f>
+        <f>Data!P17</f>
         <v>-1</v>
       </c>
       <c r="Q17" s="1">
-        <f>ROUND(Data!Q17,2)</f>
+        <f>Data!Q17</f>
         <v>-1</v>
       </c>
       <c r="R17" s="1">
-        <f>ROUND(Data!R17,2)</f>
+        <f>Data!R17</f>
         <v>-1</v>
       </c>
       <c r="S17" s="1">
-        <f>ROUND(Data!S17,2)</f>
+        <f>Data!S17</f>
         <v>-1</v>
       </c>
       <c r="T17" s="1">
-        <f>ROUND(Data!T17,2)</f>
+        <f>Data!T17</f>
         <v>-1</v>
       </c>
       <c r="U17" s="1">
-        <f>ROUND(Data!U17,2)</f>
+        <f>Data!U17</f>
         <v>-1</v>
       </c>
       <c r="V17" t="str">
@@ -6242,10 +6242,10 @@
       <c r="F20">
         <v>361</v>
       </c>
-      <c r="G20">
-        <v>-1</v>
-      </c>
-      <c r="H20">
+      <c r="G20" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H20" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6259,10 +6259,10 @@
       <c r="F21">
         <v>361</v>
       </c>
-      <c r="G21">
-        <v>-1</v>
-      </c>
-      <c r="H21">
+      <c r="G21" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H21" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6276,10 +6276,10 @@
       <c r="F22">
         <v>361</v>
       </c>
-      <c r="G22">
-        <v>-1</v>
-      </c>
-      <c r="H22">
+      <c r="G22" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H22" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6293,10 +6293,10 @@
       <c r="F23">
         <v>361</v>
       </c>
-      <c r="G23">
-        <v>-1</v>
-      </c>
-      <c r="H23">
+      <c r="G23" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H23" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6310,10 +6310,10 @@
       <c r="F24">
         <v>361</v>
       </c>
-      <c r="G24">
-        <v>-1</v>
-      </c>
-      <c r="H24">
+      <c r="G24" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H24" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6327,10 +6327,10 @@
       <c r="F25">
         <v>361</v>
       </c>
-      <c r="G25">
-        <v>-1</v>
-      </c>
-      <c r="H25">
+      <c r="G25" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H25" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6344,10 +6344,10 @@
       <c r="F26">
         <v>361</v>
       </c>
-      <c r="G26">
-        <v>-1</v>
-      </c>
-      <c r="H26">
+      <c r="G26" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H26" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6361,10 +6361,10 @@
       <c r="F27">
         <v>361</v>
       </c>
-      <c r="G27">
-        <v>-1</v>
-      </c>
-      <c r="H27">
+      <c r="G27" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H27" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6378,10 +6378,10 @@
       <c r="F28">
         <v>361</v>
       </c>
-      <c r="G28">
-        <v>-1</v>
-      </c>
-      <c r="H28">
+      <c r="G28" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H28" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6395,10 +6395,10 @@
       <c r="F29">
         <v>361</v>
       </c>
-      <c r="G29">
-        <v>-1</v>
-      </c>
-      <c r="H29">
+      <c r="G29" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H29" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6412,10 +6412,10 @@
       <c r="F30">
         <v>361</v>
       </c>
-      <c r="G30">
-        <v>-1</v>
-      </c>
-      <c r="H30">
+      <c r="G30" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H30" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6429,10 +6429,10 @@
       <c r="F31">
         <v>361</v>
       </c>
-      <c r="G31">
-        <v>-1</v>
-      </c>
-      <c r="H31">
+      <c r="G31" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H31" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6446,10 +6446,10 @@
       <c r="F32">
         <v>361</v>
       </c>
-      <c r="G32">
-        <v>-1</v>
-      </c>
-      <c r="H32">
+      <c r="G32" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H32" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6463,10 +6463,10 @@
       <c r="F33">
         <v>361</v>
       </c>
-      <c r="G33">
-        <v>-1</v>
-      </c>
-      <c r="H33">
+      <c r="G33" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H33" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -6480,10 +6480,10 @@
       <c r="F34">
         <v>361</v>
       </c>
-      <c r="G34">
-        <v>-1</v>
-      </c>
-      <c r="H34">
+      <c r="G34" s="1">
+        <v>-1</v>
+      </c>
+      <c r="H34" s="1">
         <v>-1</v>
       </c>
     </row>
@@ -7145,10 +7145,10 @@
         <f>MAX(MAX(J14:J19)-MIN(J14:J19),MAX(K14:K19)-MIN(K14:K19))</f>
         <v>#VALUE!</v>
       </c>
-      <c r="O12" s="45" t="s">
+      <c r="O12" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="P12" s="45"/>
+      <c r="P12" s="46"/>
       <c r="Q12" s="13" t="s">
         <v>79</v>
       </c>
@@ -7677,30 +7677,30 @@
       <c r="U20" s="1"/>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="L21" s="41" t="s">
+      <c r="L21" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="M21" s="42"/>
-      <c r="P21" s="41" t="s">
+      <c r="M21" s="43"/>
+      <c r="P21" s="42" t="s">
         <v>81</v>
       </c>
-      <c r="Q21" s="42"/>
-      <c r="R21" s="41" t="s">
+      <c r="Q21" s="43"/>
+      <c r="R21" s="42" t="s">
         <v>82</v>
       </c>
-      <c r="S21" s="42"/>
+      <c r="S21" s="43"/>
     </row>
     <row r="22" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f>Data!A19</f>
         <v>ballCBCT</v>
       </c>
-      <c r="L22" s="43"/>
-      <c r="M22" s="44"/>
-      <c r="P22" s="43"/>
-      <c r="Q22" s="44"/>
-      <c r="R22" s="43"/>
-      <c r="S22" s="44"/>
+      <c r="L22" s="44"/>
+      <c r="M22" s="45"/>
+      <c r="P22" s="44"/>
+      <c r="Q22" s="45"/>
+      <c r="R22" s="44"/>
+      <c r="S22" s="45"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
@@ -7790,12 +7790,12 @@
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="H2" s="46" t="s">
+      <c r="H2" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
       <c r="L2" s="35">
         <f>MAX(L4:L6)</f>
         <v>0</v>

</xml_diff>